<commit_message>
add lead management, update selenium version 3 to 4, add mobile config
</commit_message>
<xml_diff>
--- a/testdata/CallScheduller.xlsx
+++ b/testdata/CallScheduller.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8F8337-91CD-4FBA-99D7-0247B092BFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{894085D5-DED7-4C7C-AE32-F67D622939A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="31">
   <si>
     <t>Create task succesfully</t>
   </si>
@@ -118,6 +118,15 @@
   </si>
   <si>
     <t>Cabang Pondok Indah</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Cabang Kebayoran Lama</t>
+  </si>
+  <si>
+    <t>Penjualan product dari cabang outlet Kebayoran Lama</t>
   </si>
 </sst>
 </file>
@@ -492,7 +501,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E5AD2E2-3C9A-4FB7-87F8-04A08F84B4E2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -565,28 +574,28 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
         <v>0</v>
@@ -600,22 +609,22 @@
         <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I4" t="s">
         <v>0</v>
@@ -626,27 +635,56 @@
         <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="E5" t="s">
         <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H5" t="s">
         <v>24</v>
       </c>
       <c r="I5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix bug and tidy up code
</commit_message>
<xml_diff>
--- a/testdata/CallScheduller.xlsx
+++ b/testdata/CallScheduller.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{894085D5-DED7-4C7C-AE32-F67D622939A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6824486E-CC7B-4313-B5CB-3472FC6B57CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
@@ -511,7 +511,7 @@
     <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="54.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add mobile automation & fix issue
</commit_message>
<xml_diff>
--- a/testdata/CallScheduller.xlsx
+++ b/testdata/CallScheduller.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6824486E-CC7B-4313-B5CB-3472FC6B57CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664BFBA9-7BC5-4706-B9C3-A5B44CB069EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Create task succesfully</t>
   </si>
@@ -96,37 +96,16 @@
     <t>10:00AM</t>
   </si>
   <si>
-    <t>Cabang Permata Hijau</t>
-  </si>
-  <si>
     <t>Buying</t>
   </si>
   <si>
-    <t>Santi Nurmala</t>
-  </si>
-  <si>
-    <t>Penjualan product dari cabang outlet green garden</t>
-  </si>
-  <si>
-    <t>Penjualan product dari cabang outlet permata hijau</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>Suka Makmur</t>
   </si>
   <si>
     <t>Cabang Pondok Indah</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Cabang Kebayoran Lama</t>
-  </si>
-  <si>
-    <t>Penjualan product dari cabang outlet Kebayoran Lama</t>
+    <t>Penjualan product dari cabang outlet pondok hijau</t>
   </si>
 </sst>
 </file>
@@ -501,7 +480,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E5AD2E2-3C9A-4FB7-87F8-04A08F84B4E2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -586,105 +565,18 @@
         <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>